<commit_message>
chore(brand/templates): regenerate the two config workbooks
Brand_Config_Template.xlsx is what an analyst copies into a new project, so
the new fieldwork_dates Settings key had to reach it.

Regenerated with generate_brand_templates("modules/brand/templates",
overwrite = TRUE) from the worktree root, which saves through
turas_saveWorkbook. Read back against a snapshot taken first: Settings goes
from 79 rows to 81, adding fieldwork_dates and funnel_consideration_roles.
The second is not this branch's work. It was added to the generator by the
funnel definition change on 6 September and the template was never
regenerated, so that drift is corrected here as a side effect.

Nothing was removed, the three sheets are unchanged, the dropdown count is 15
before and after, and neither workbook references a drawing part.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/brand/templates/Brand_Config_Template.xlsx
+++ b/modules/brand/templates/Brand_Config_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="264">
   <si>
     <t xml:space="preserve">TURAS Brand Module: Configuration</t>
   </si>
@@ -112,6 +112,15 @@
     <t xml:space="preserve">Integer &gt;= 1</t>
   </si>
   <si>
+    <t xml:space="preserve">fieldwork_dates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When this wave was in field, in your own words. Shown in the report header next to the wave and on the About tab. Leave blank and the header shows only the date the report was generated, which is not the study's date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free text (e.g. '19 to 26 May 2026')</t>
+  </si>
+  <si>
     <t xml:space="preserve">respondent_id_col</t>
   </si>
   <si>
@@ -362,6 +371,15 @@
   </si>
   <si>
     <t xml:space="preserve">Attitude option code (e.g. 4), or blank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funnel_consideration_roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which positions on the brand attitude scale count as consideration. Named by role, never by response code, so the definition survives a survey that exports labels rather than numbers. Comma separated. Leave blank for the Turas standard. Valid roles: love, prefer, ambivalent, price, avoid, no_opinion. A role named here that the scale does not carry refuses the run rather than returning an empty stage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comma separated roles (e.g. love, prefer, price), or blank</t>
   </si>
   <si>
     <t xml:space="preserve">DRIVERS &amp; BARRIERS OPTIONS  (only if element_drivers_barriers = Y)</t>
@@ -1467,27 +1485,27 @@
         <v>32</v>
       </c>
       <c r="B13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="14" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>15</v>
+      <c r="C14" s="16" t="s">
+        <v>4</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>37</v>
@@ -1497,57 +1515,57 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
+      <c r="B15" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="14" t="s">
+      <c r="A16" s="9" t="s">
         <v>42</v>
       </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>15</v>
       </c>
       <c r="D17" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="14" t="s">
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="s">
+      <c r="B18" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>4</v>
+      <c r="C18" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>48</v>
@@ -1557,71 +1575,71 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
+      <c r="B19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="12" t="s">
+      <c r="A20" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B21" s="11" t="s">
+      <c r="D21" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="13" t="s">
+      <c r="E21" s="14" t="s">
         <v>57</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="C22" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22" s="13" t="s">
+      <c r="E22" s="14" t="s">
         <v>61</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>63</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>4</v>
@@ -1630,177 +1648,177 @@
         <v>64</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>62</v>
-      </c>
+      <c r="A25" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
     </row>
     <row r="26">
       <c r="A26" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>4</v>
@@ -1809,7 +1827,7 @@
         <v>86</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35">
@@ -1817,67 +1835,67 @@
         <v>87</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
+      <c r="A37" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="B38" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E38" s="14" t="s">
+      <c r="A38" s="9" t="s">
         <v>94</v>
       </c>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="s">
         <v>95</v>
       </c>
       <c r="B39" s="11" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C39" s="12" t="s">
         <v>15</v>
@@ -1890,54 +1908,54 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="15" t="s">
+      <c r="A40" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="C40" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D40" s="13" t="s">
+      <c r="E40" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="E40" s="14" t="s">
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="s">
+      <c r="B41" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B41" s="9"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
+      <c r="C41" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="s">
-        <v>103</v>
-      </c>
-      <c r="B42" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D42" s="13" t="s">
+      <c r="A42" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="E42" s="14" t="s">
-        <v>106</v>
-      </c>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
     </row>
     <row r="43">
       <c r="A43" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" s="11" t="s">
         <v>107</v>
-      </c>
-      <c r="B43" s="11" t="n">
-        <v>75</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>4</v>
@@ -1954,7 +1972,7 @@
         <v>110</v>
       </c>
       <c r="B44" s="11" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C44" s="16" t="s">
         <v>4</v>
@@ -1970,8 +1988,8 @@
       <c r="A45" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="B45" s="11" t="s">
-        <v>14</v>
+      <c r="B45" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="C45" s="16" t="s">
         <v>4</v>
@@ -1984,34 +2002,42 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
+      <c r="B46" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="15" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="C47" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>62</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" s="9"/>
@@ -2020,44 +2046,36 @@
     </row>
     <row r="49">
       <c r="A49" s="15" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>123</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="B50" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C50" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D50" s="13" t="s">
+      <c r="A50" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E50" s="14" t="s">
-        <v>126</v>
-      </c>
+      <c r="B50" s="9"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
     </row>
     <row r="51">
       <c r="A51" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B51" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="B51" s="11" t="n">
-        <v>0.5</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>4</v>
@@ -2066,15 +2084,15 @@
         <v>128</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="B52" s="11" t="s">
         <v>130</v>
+      </c>
+      <c r="B52" s="11" t="n">
+        <v>0.5</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>4</v>
@@ -2087,71 +2105,71 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="s">
+      <c r="A53" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
+      <c r="B53" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>14</v>
+        <v>136</v>
       </c>
       <c r="C54" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="B55" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C55" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D55" s="13" t="s">
+      <c r="A55" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="E55" s="14" t="s">
-        <v>140</v>
-      </c>
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
     </row>
     <row r="56">
       <c r="A56" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="C56" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D56" s="13" t="s">
+      <c r="E56" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="E56" s="14" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="B57" s="11" t="s">
         <v>144</v>
-      </c>
-      <c r="B57" s="11" t="n">
-        <v>20</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>4</v>
@@ -2167,48 +2185,56 @@
       <c r="A58" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="C58" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D58" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="C58" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D58" s="13" t="s">
+      <c r="E58" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="E58" s="14" t="s">
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="s">
+      <c r="B59" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="C59" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
+      <c r="E59" s="14" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="B60" s="11" t="n">
-        <v>6</v>
+        <v>153</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>154</v>
       </c>
       <c r="C60" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E60" s="14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
@@ -2217,44 +2243,36 @@
     </row>
     <row r="62">
       <c r="A62" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B62" s="11" t="n">
-        <v>0.05</v>
+        <v>6</v>
       </c>
       <c r="C62" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="B63" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C63" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D63" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="E63" s="14" t="s">
+      <c r="A63" s="9" t="s">
         <v>161</v>
       </c>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
     </row>
     <row r="64">
       <c r="A64" s="15" t="s">
         <v>162</v>
       </c>
       <c r="B64" s="11" t="n">
-        <v>30</v>
+        <v>0.05</v>
       </c>
       <c r="C64" s="16" t="s">
         <v>4</v>
@@ -2263,246 +2281,280 @@
         <v>163</v>
       </c>
       <c r="E64" s="14" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="B65" s="11" t="n">
-        <v>75</v>
+        <v>165</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C65" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E65" s="14" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
+      <c r="A66" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B66" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="C66" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D66" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E66" s="14" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B67" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
+      </c>
+      <c r="B67" s="11" t="n">
+        <v>75</v>
       </c>
       <c r="C67" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E67" s="14" t="s">
-        <v>170</v>
+        <v>112</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="B68" s="11" t="s">
+      <c r="A68" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C68" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D68" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="E68" s="14" t="s">
-        <v>174</v>
-      </c>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
     </row>
     <row r="69">
       <c r="A69" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C69" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D69" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="E69" s="14" t="s">
         <v>176</v>
-      </c>
-      <c r="C69" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D69" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="E69" s="14" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="B70" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="C70" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D70" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="C70" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D70" s="13" t="s">
+      <c r="E70" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="E70" s="14" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="71">
-      <c r="A71" s="9" t="s">
+      <c r="A71" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
+      <c r="B71" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="E71" s="14" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="s">
-        <v>182</v>
+      <c r="A72" s="15" t="s">
+        <v>184</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="C72" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="C72" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D72" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="C74" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D72" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="E72" s="14" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="B73" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C73" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D73" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="E73" s="14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="B74" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C74" s="16" t="s">
-        <v>4</v>
-      </c>
       <c r="D74" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>62</v>
+        <v>191</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="15" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C75" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E75" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="B76" s="11" t="n">
-        <v>0</v>
+        <v>194</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>63</v>
       </c>
       <c r="C76" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>194</v>
+        <v>65</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C77" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E77" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="B78" s="11" t="s">
-        <v>60</v>
+        <v>198</v>
+      </c>
+      <c r="B78" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="C78" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E78" s="14" t="s">
-        <v>62</v>
+        <v>200</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="15" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>200</v>
+        <v>63</v>
       </c>
       <c r="C79" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E79" s="14" t="s">
-        <v>202</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C80" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="E80" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C81" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E81" s="14" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2510,73 +2562,73 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A73:E73"/>
   </mergeCells>
   <dataValidations count="14">
     <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B12:B12">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B38:B38">
+    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B39:B39">
       <formula1>1</formula1>
       <formula2>24</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B39:B39">
+    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B40:B40">
       <formula1>2</formula1>
       <formula2>36</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B43:B43">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B44:B44">
       <formula1>30</formula1>
       <formula2>500</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B44:B44">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B45:B45">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B50:B50">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B52:B52">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B51:B51">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B53:B53">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B56:B56">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B58:B58">
       <formula1>10</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B57:B57">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B59:B59">
       <formula1>5</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B60:B60">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B62:B62">
       <formula1>2</formula1>
       <formula2>8</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B62:B62">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B64:B64">
       <formula1>0.01</formula1>
       <formula2>0.2</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B64:B64">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B66:B66">
       <formula1>10</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B65:B65">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B67:B67">
       <formula1>30</formula1>
       <formula2>500</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B76:B76">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B78:B78">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
@@ -2596,13 +2648,7 @@
           <x14:formula1>
             <xm:f>"balanced,quota,priority"</xm:f>
           </x14:formula1>
-          <xm:sqref>B20:B20</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>"Y,N"</xm:f>
-          </x14:formula1>
-          <xm:sqref>B22:B22</xm:sqref>
+          <xm:sqref>B21:B21</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -2614,7 +2660,7 @@
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B25:B25</xm:sqref>
+          <xm:sqref>B24:B24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -2684,51 +2730,45 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
+            <xm:f>"Y,N"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B37:B37</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
             <xm:f>"ratio,absolute"</xm:f>
           </x14:formula1>
-          <xm:sqref>B42:B42</xm:sqref>
+          <xm:sqref>B43:B43</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B47:B47</xm:sqref>
+          <xm:sqref>B49:B49</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"brand,category"</xm:f>
           </x14:formula1>
-          <xm:sqref>B49:B49</xm:sqref>
+          <xm:sqref>B51:B51</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"open,closed_list"</xm:f>
           </x14:formula1>
-          <xm:sqref>B52:B52</xm:sqref>
+          <xm:sqref>B54:B54</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"3m,13m"</xm:f>
           </x14:formula1>
-          <xm:sqref>B55:B55</xm:sqref>
+          <xm:sqref>B57:B57</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"all,non_buyers"</xm:f>
           </x14:formula1>
-          <xm:sqref>B58:B58</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>"Y,N"</xm:f>
-          </x14:formula1>
-          <xm:sqref>B73:B73</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>"Y,N"</xm:f>
-          </x14:formula1>
-          <xm:sqref>B74:B74</xm:sqref>
+          <xm:sqref>B60:B60</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -2740,19 +2780,31 @@
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
+          <xm:sqref>B76:B76</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Y,N"</xm:f>
+          </x14:formula1>
           <xm:sqref>B77:B77</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B78:B78</xm:sqref>
+          <xm:sqref>B79:B79</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Y,N"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B80:B80</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"focal_only,all"</xm:f>
           </x14:formula1>
-          <xm:sqref>B79:B79</xm:sqref>
+          <xm:sqref>B81:B81</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2778,93 +2830,93 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H5" s="17" t="n">
         <v>0.25</v>
@@ -2875,25 +2927,25 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H6" s="17" t="n">
         <v>0.25</v>
@@ -2904,25 +2956,25 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B7" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="C7" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>225</v>
-      </c>
       <c r="E7" s="17" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H7" s="17" t="n">
         <v>0.25</v>
@@ -2933,25 +2985,25 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B8" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="F8" s="17" t="s">
         <v>233</v>
       </c>
-      <c r="C8" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>225</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>227</v>
-      </c>
       <c r="G8" s="17" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H8" s="17" t="n">
         <v>0.25</v>
@@ -3145,79 +3197,79 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>14</v>
@@ -3225,16 +3277,16 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9">

</xml_diff>